<commit_message>
fix in game dds
</commit_message>
<xml_diff>
--- a/data/mpg/mpg_round3_top5_bets.xlsx
+++ b/data/mpg/mpg_round3_top5_bets.xlsx
@@ -129,45 +129,45 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Draw</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>0-0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="H2">
-        <v>0.4033014374680687</v>
+        <v>0.5092867836944935</v>
       </c>
       <c r="I2">
-        <v>108.0</v>
+        <v>96.0</v>
       </c>
       <c r="J2">
-        <v>43.55655524655142</v>
+        <v>48.891531234671376</v>
       </c>
       <c r="K2">
-        <v>0.3034148547376874</v>
+        <v>0.11055701804772465</v>
       </c>
       <c r="L2">
-        <v>0.7508755811175876</v>
+        <v>0.21694311728211282</v>
       </c>
       <c r="M2">
-        <v>0.8282858904878876</v>
+        <v>0.17955358356768283</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Exact</t>
+          <t>Tres rare</t>
         </is>
       </c>
       <c r="O2">
-        <v>20.0</v>
+        <v>50.0</v>
       </c>
       <c r="P2">
-        <v>6.068297094753748</v>
+        <v>5.527850902386232</v>
       </c>
       <c r="Q2">
-        <v>49.624852341305164</v>
+        <v>54.41938213705761</v>
       </c>
     </row>
     <row r="3">
@@ -196,31 +196,31 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Draw</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>1-1</t>
+          <t>2-0</t>
         </is>
       </c>
       <c r="H3">
-        <v>0.4033014374680687</v>
+        <v>0.5092867836944935</v>
       </c>
       <c r="I3">
-        <v>108.0</v>
+        <v>96.0</v>
       </c>
       <c r="J3">
-        <v>43.55655524655142</v>
+        <v>48.891531234671376</v>
       </c>
       <c r="K3">
-        <v>0.09260282764414957</v>
+        <v>0.09963162213064454</v>
       </c>
       <c r="L3">
-        <v>0.2291687467989873</v>
+        <v>0.1955045013566229</v>
       </c>
       <c r="M3">
-        <v>0.15556586453121213</v>
+        <v>0.18203608413450684</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -231,10 +231,10 @@
         <v>50.0</v>
       </c>
       <c r="P3">
-        <v>4.630141382207478</v>
+        <v>4.981581106532227</v>
       </c>
       <c r="Q3">
-        <v>48.186696628758895</v>
+        <v>53.8731123412036</v>
       </c>
     </row>
     <row r="4">
@@ -263,45 +263,45 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Draw</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2-2</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="H4">
-        <v>0.4033014374680687</v>
+        <v>0.5092867836944935</v>
       </c>
       <c r="I4">
-        <v>108.0</v>
+        <v>96.0</v>
       </c>
       <c r="J4">
-        <v>43.55655524655142</v>
+        <v>48.891531234671376</v>
       </c>
       <c r="K4">
-        <v>0.007432744453083944</v>
+        <v>0.09695442895789146</v>
       </c>
       <c r="L4">
-        <v>0.01839417623548114</v>
+        <v>0.19025111588440685</v>
       </c>
       <c r="M4">
-        <v>0.0156080724814215</v>
+        <v>0.29524101233389566</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Mega rare</t>
+          <t>Rare</t>
         </is>
       </c>
       <c r="O4">
-        <v>70.0</v>
+        <v>30.0</v>
       </c>
       <c r="P4">
-        <v>0.5202921117158761</v>
+        <v>2.9086328687367438</v>
       </c>
       <c r="Q4">
-        <v>44.076847358267294</v>
+        <v>51.80016410340812</v>
       </c>
     </row>
     <row r="5">
@@ -330,45 +330,45 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Draw</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>3-3</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H5">
-        <v>0.4033014374680687</v>
+        <v>0.5092867836944935</v>
       </c>
       <c r="I5">
-        <v>108.0</v>
+        <v>96.0</v>
       </c>
       <c r="J5">
-        <v>43.55655524655142</v>
+        <v>48.891531234671376</v>
       </c>
       <c r="K5">
-        <v>0.0006228917335824087</v>
+        <v>0.03673263369164942</v>
       </c>
       <c r="L5">
-        <v>0.0015415006388905632</v>
+        <v>0.07207947717627859</v>
       </c>
       <c r="M5">
-        <v>0.0005232058972133063</v>
+        <v>0.03728548925297283</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Ultra rare</t>
+          <t>Mega rare</t>
         </is>
       </c>
       <c r="O5">
-        <v>100.0</v>
+        <v>70.0</v>
       </c>
       <c r="P5">
-        <v>0.062289173358240864</v>
+        <v>2.5712843584154594</v>
       </c>
       <c r="Q5">
-        <v>43.61884441990966</v>
+        <v>51.46281559308684</v>
       </c>
     </row>
     <row r="6">
@@ -397,45 +397,45 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Draw</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>4-4</t>
+          <t>4-1</t>
         </is>
       </c>
       <c r="H6">
-        <v>0.4033014374680687</v>
+        <v>0.5092867836944935</v>
       </c>
       <c r="I6">
-        <v>108.0</v>
+        <v>96.0</v>
       </c>
       <c r="J6">
-        <v>43.55655524655142</v>
+        <v>48.891531234671376</v>
       </c>
       <c r="K6">
-        <v>7.894543154473964e-06</v>
+        <v>0.031889547849941094</v>
       </c>
       <c r="L6">
-        <v>1.9537012068503745e-05</v>
+        <v>0.0625760177096754</v>
       </c>
       <c r="M6">
-        <v>1.6577806830371323e-05</v>
+        <v>0.03236951108984722</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Ultra rare</t>
+          <t>Mega rare</t>
         </is>
       </c>
       <c r="O6">
-        <v>100.0</v>
+        <v>70.0</v>
       </c>
       <c r="P6">
-        <v>0.0007894543154473964</v>
+        <v>2.2322683494958766</v>
       </c>
       <c r="Q6">
-        <v>43.557344700866864</v>
+        <v>51.12379958416725</v>
       </c>
     </row>
     <row r="7">
@@ -473,22 +473,22 @@
         </is>
       </c>
       <c r="H7">
-        <v>0.967577190262213</v>
+        <v>0.8686669773038992</v>
       </c>
       <c r="I7">
         <v>56.0</v>
       </c>
       <c r="J7">
-        <v>54.184322654683925</v>
+        <v>48.645350729018354</v>
       </c>
       <c r="K7">
-        <v>0.16682026612393575</v>
+        <v>0.17800937997727778</v>
       </c>
       <c r="L7">
-        <v>0.18016441107145345</v>
+        <v>0.20254170078674147</v>
       </c>
       <c r="M7">
-        <v>0.1619452409691271</v>
+        <v>0.1828398700353069</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
@@ -499,10 +499,10 @@
         <v>50.0</v>
       </c>
       <c r="P7">
-        <v>8.341013306196787</v>
+        <v>8.90046899886389</v>
       </c>
       <c r="Q7">
-        <v>62.52533596088071</v>
+        <v>57.54581972788225</v>
       </c>
     </row>
     <row r="8">
@@ -540,22 +540,22 @@
         </is>
       </c>
       <c r="H8">
-        <v>0.967577190262213</v>
+        <v>0.8686669773038992</v>
       </c>
       <c r="I8">
         <v>56.0</v>
       </c>
       <c r="J8">
-        <v>54.184322654683925</v>
+        <v>48.645350729018354</v>
       </c>
       <c r="K8">
-        <v>0.129443404039074</v>
+        <v>0.12002009852278538</v>
       </c>
       <c r="L8">
-        <v>0.1397977308012327</v>
+        <v>0.13656064015559286</v>
       </c>
       <c r="M8">
-        <v>0.15358524024185327</v>
+        <v>0.15067186746729072</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
@@ -566,10 +566,10 @@
         <v>50.0</v>
       </c>
       <c r="P8">
-        <v>6.4721702019537</v>
+        <v>6.001004926139268</v>
       </c>
       <c r="Q8">
-        <v>60.65649285663763</v>
+        <v>54.64635565515762</v>
       </c>
     </row>
     <row r="9">
@@ -603,26 +603,26 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>0-4</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="H9">
-        <v>0.967577190262213</v>
+        <v>0.8686669773038992</v>
       </c>
       <c r="I9">
         <v>56.0</v>
       </c>
       <c r="J9">
-        <v>54.184322654683925</v>
+        <v>48.645350729018354</v>
       </c>
       <c r="K9">
-        <v>0.09002251880787042</v>
+        <v>0.0864245050353621</v>
       </c>
       <c r="L9">
-        <v>0.0972235236223598</v>
+        <v>0.0983350778579698</v>
       </c>
       <c r="M9">
-        <v>0.11652236137910156</v>
+        <v>0.147949556277581</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
@@ -633,10 +633,10 @@
         <v>50.0</v>
       </c>
       <c r="P9">
-        <v>4.501125940393521</v>
+        <v>4.321225251768105</v>
       </c>
       <c r="Q9">
-        <v>58.685448595077446</v>
+        <v>52.96657598078646</v>
       </c>
     </row>
     <row r="10">
@@ -670,26 +670,26 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="H10">
-        <v>0.967577190262213</v>
+        <v>0.8686669773038992</v>
       </c>
       <c r="I10">
         <v>56.0</v>
       </c>
       <c r="J10">
-        <v>54.184322654683925</v>
+        <v>48.645350729018354</v>
       </c>
       <c r="K10">
-        <v>0.0641710214370617</v>
+        <v>0.07545589839142147</v>
       </c>
       <c r="L10">
-        <v>0.0693041352450102</v>
+        <v>0.08585483527070802</v>
       </c>
       <c r="M10">
-        <v>0.10382622938369798</v>
+        <v>0.06889198339271474</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
@@ -700,10 +700,10 @@
         <v>50.0</v>
       </c>
       <c r="P10">
-        <v>3.208551071853085</v>
+        <v>3.7727949195710737</v>
       </c>
       <c r="Q10">
-        <v>57.39287372653701</v>
+        <v>52.41814564858943</v>
       </c>
     </row>
     <row r="11">
@@ -737,26 +737,26 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>0-4</t>
         </is>
       </c>
       <c r="H11">
-        <v>0.967577190262213</v>
+        <v>0.8686669773038992</v>
       </c>
       <c r="I11">
         <v>56.0</v>
       </c>
       <c r="J11">
-        <v>54.184322654683925</v>
+        <v>48.645350729018354</v>
       </c>
       <c r="K11">
-        <v>0.06144394507410913</v>
+        <v>0.07252791449382026</v>
       </c>
       <c r="L11">
-        <v>0.06635891690737</v>
+        <v>0.08252333196132039</v>
       </c>
       <c r="M11">
-        <v>0.053020760192704644</v>
+        <v>0.09932805759392878</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
@@ -767,10 +767,10 @@
         <v>50.0</v>
       </c>
       <c r="P11">
-        <v>3.0721972537054563</v>
+        <v>3.626395724691013</v>
       </c>
       <c r="Q11">
-        <v>57.25651990838938</v>
+        <v>52.27174645370937</v>
       </c>
     </row>
     <row r="12">

</xml_diff>